<commit_message>
docs: update customer responses and statuses in Open Questions documentation
</commit_message>
<xml_diff>
--- a/Ansible to Orchestrator Transition/Ansible to Orchestrator Projects.xlsx
+++ b/Ansible to Orchestrator Transition/Ansible to Orchestrator Projects.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\GitHub-LocalRepos\AutomationProjects\Ansible to Orchestrator Transition\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ForgusonJW\Documents\GitHubRepos\Ansible to Orchestrator Transition\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74A23DD3-0757-4D22-A7A3-352C8DEF1E8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{127D4597-EAE3-460E-8389-062ACC168E5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5595" yWindow="2925" windowWidth="44085" windowHeight="17730" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Consolidated Playbooks" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Add PowerShell script and Ansible playbook for managing pending reboots
- Created Set-PendingRebootFlag.ps1 to set, clear, or check pending reboot registry keys for testing purposes.
- Added servers_reboot.yml playbook to execute PowerShell script remotely on specified hosts.
- Introduced vars.txt for configurable variables related to the PowerShell script execution and email reporting.
</commit_message>
<xml_diff>
--- a/Ansible to Orchestrator Transition/Ansible to Orchestrator Projects.xlsx
+++ b/Ansible to Orchestrator Transition/Ansible to Orchestrator Projects.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\GitHub-LocalRepos\AutomationProjects\Ansible to Orchestrator Transition\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49F87C17-6E1C-4683-AFF5-6C1E59D5CBE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C09C01B3-2F51-45FA-B3AA-281118C41FB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10335" yWindow="6525" windowWidth="34905" windowHeight="12300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Consolidated Playbooks" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,6 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Consolidated Playbooks'!$C$1:$X$65</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -40,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1031" uniqueCount="595">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1032" uniqueCount="595">
   <si>
     <t>Rank</t>
   </si>
@@ -4261,7 +4260,9 @@
         <v>200</v>
       </c>
       <c r="F9" s="8"/>
-      <c r="G9" s="8"/>
+      <c r="G9" s="8" t="s">
+        <v>594</v>
+      </c>
       <c r="H9" s="8"/>
       <c r="I9" s="8" t="s">
         <v>93</v>
@@ -8170,18 +8171,18 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -8203,18 +8204,18 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4C681E44-B091-4BF0-A8C6-EEF41310CEFC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B266BC6E-C493-4766-9D5B-54989D07BF17}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4C681E44-B091-4BF0-A8C6-EEF41310CEFC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
feat: Update Ansible to Orchestrator Projects.xlsx and remove temporary file
</commit_message>
<xml_diff>
--- a/Ansible to Orchestrator Transition/Ansible to Orchestrator Projects.xlsx
+++ b/Ansible to Orchestrator Transition/Ansible to Orchestrator Projects.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\GitHub-LocalRepos\AutomationProjects\Ansible to Orchestrator Transition\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{172F47FC-4413-4473-96CE-8DB3F6715DCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A05B0D7-0513-4B72-AD27-80107716C145}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9780" yWindow="1380" windowWidth="41340" windowHeight="17445" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4680" yWindow="4140" windowWidth="30075" windowHeight="13095" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Consolidated Playbooks" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1034" uniqueCount="595">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1038" uniqueCount="596">
   <si>
     <t>Rank</t>
   </si>
@@ -3183,6 +3183,9 @@
   </si>
   <si>
     <t>Completed</t>
+  </si>
+  <si>
+    <t>In progress</t>
   </si>
 </sst>
 </file>
@@ -4566,7 +4569,9 @@
         <v>77</v>
       </c>
       <c r="F13" s="8"/>
-      <c r="G13" s="8"/>
+      <c r="G13" s="8" t="s">
+        <v>594</v>
+      </c>
       <c r="H13" s="8"/>
       <c r="I13" s="8"/>
       <c r="J13" s="8" t="s">
@@ -4643,7 +4648,9 @@
         <v>39</v>
       </c>
       <c r="F14" s="8"/>
-      <c r="G14" s="8"/>
+      <c r="G14" s="8" t="s">
+        <v>594</v>
+      </c>
       <c r="H14" s="8"/>
       <c r="I14" s="8"/>
       <c r="J14" s="8" t="s">
@@ -4783,7 +4790,9 @@
         <v>31</v>
       </c>
       <c r="F16" s="8"/>
-      <c r="G16" s="8"/>
+      <c r="G16" s="8" t="s">
+        <v>595</v>
+      </c>
       <c r="H16" s="8"/>
       <c r="I16" s="8"/>
       <c r="J16" s="8" t="s">
@@ -5057,7 +5066,9 @@
         <v>16</v>
       </c>
       <c r="F20" s="8"/>
-      <c r="G20" s="8"/>
+      <c r="G20" s="8" t="s">
+        <v>594</v>
+      </c>
       <c r="H20" s="8"/>
       <c r="I20" s="8"/>
       <c r="J20" s="8" t="s">
@@ -8175,18 +8186,18 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -8208,18 +8219,18 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4C681E44-B091-4BF0-A8C6-EEF41310CEFC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B266BC6E-C493-4766-9D5B-54989D07BF17}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4C681E44-B091-4BF0-A8C6-EEF41310CEFC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Add Platform Options Advisory for Datastore Capacity and Fill Projection
This advisory outlines the recommendation for VCF Operations to manage datastore fill projections and alerting, rather than transitioning the existing PowerShell script to Orchestrator. It details the capabilities of VCF Operations, the advantages of using its native features, and the implications for reporting and alerting. The document also includes validation steps before retiring the existing script and clarifies the impact on the current deliverable.
</commit_message>
<xml_diff>
--- a/Ansible to Orchestrator Transition/Ansible to Orchestrator Projects.xlsx
+++ b/Ansible to Orchestrator Transition/Ansible to Orchestrator Projects.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\GitHub-LocalRepos\AutomationProjects\Ansible to Orchestrator Transition\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A05B0D7-0513-4B72-AD27-80107716C145}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{059695C4-73AB-454A-B5C7-D0E3CCC7FD1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4680" yWindow="4140" windowWidth="30075" windowHeight="13095" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11175" yWindow="6060" windowWidth="22560" windowHeight="11655" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Consolidated Playbooks" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1038" uniqueCount="596">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1041" uniqueCount="597">
   <si>
     <t>Rank</t>
   </si>
@@ -3185,7 +3185,10 @@
     <t>Completed</t>
   </si>
   <si>
-    <t>In progress</t>
+    <t>Will use VCF Operations reports</t>
+  </si>
+  <si>
+    <t>In Progress</t>
   </si>
 </sst>
 </file>
@@ -4791,7 +4794,7 @@
       </c>
       <c r="F16" s="8"/>
       <c r="G16" s="8" t="s">
-        <v>595</v>
+        <v>109</v>
       </c>
       <c r="H16" s="8"/>
       <c r="I16" s="8"/>
@@ -4859,8 +4862,12 @@
         <v>29</v>
       </c>
       <c r="F17" s="8"/>
-      <c r="G17" s="8"/>
-      <c r="H17" s="8"/>
+      <c r="G17" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="H17" s="8" t="s">
+        <v>595</v>
+      </c>
       <c r="I17" s="8"/>
       <c r="J17" s="8" t="s">
         <v>34</v>
@@ -4999,7 +5006,9 @@
         <v>18</v>
       </c>
       <c r="F19" s="8"/>
-      <c r="G19" s="8"/>
+      <c r="G19" s="8" t="s">
+        <v>596</v>
+      </c>
       <c r="H19" s="8"/>
       <c r="I19" s="8"/>
       <c r="J19" s="8" t="s">
@@ -8186,18 +8195,18 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -8219,18 +8228,18 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4C681E44-B091-4BF0-A8C6-EEF41310CEFC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B266BC6E-C493-4766-9D5B-54989D07BF17}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4C681E44-B091-4BF0-A8C6-EEF41310CEFC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>